<commit_message>
docs(decisions): reconcile IDs and release scope plan
</commit_message>
<xml_diff>
--- a/docs/CONNECTSPHERE BACKLOGS CAA 181026.xlsx
+++ b/docs/CONNECTSPHERE BACKLOGS CAA 181026.xlsx
@@ -1138,7 +1138,7 @@
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Previous event copied
-Given I choose one of my own completed or past events When I copy it Then ConnectSphere creates a new draft with the event requirements and Session structure copied, all event and Session dates/times left blank, and no bookings, reservations, or registrations carried over (T-98)
+Given I choose one of my own completed or past events When I copy it Then ConnectSphere creates a new draft with the event requirements and Session structure copied, all event and Session dates/times left blank, and no bookings, reservations, or registrations carried over (T-99)
 Scenario 2 - Missing reference flagged
 Given the copied event references a venue or equipment item that no longer exists When the draft is created Then the affected requirement is flagged for review and identifies its Session rather than being copied silently
 Scenario 3 - Dates remain subject to current submission policy
@@ -1146,7 +1146,7 @@
 Checklist
 - Copy one of my own completed or past events into a new draft
 - Confirm requirements and Session structure are copied while event and Session dates/times are blank
-- Confirm bookings, equipment reservations and registrations are not copied (T-98)
+- Confirm bookings, equipment reservations and registrations are not copied (T-99)
 - See unavailable venue/equipment references flagged against the relevant Session
 - Submit a copied draft subject to the current date rules</t>
         </is>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>C-74, T-79, T-87, T-90, T-98</t>
+          <t>C-74, T-79, T-87, T-90, T-99</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr"/>
@@ -3411,7 +3411,7 @@
 Scenario 4 - Concurrent submissions do not overbook
 Given one approved seat remains in a Session or in the combined Event capacity When two registrations are submitted at the same time Then at most one is confirmed against that remaining capacity and any other submission that exceeds capacity is Pending
 Scenario 5 - Waiting list remains event-level
-Given the combined Event capacity is full When an Attendee opens registration Then the existing Event-level waiting-list option is offered where enabled; a full selected Session follows the Pending decision path and has no separate Session-level waiting list (T-97)
+Given the combined Event capacity is full When an Attendee opens registration Then the existing Event-level waiting-list option is offered where enabled; a full selected Session follows the Pending decision path and has no separate Session-level waiting list (T-98)
 Scenario 6 - Manual addition allowed within both limits
 Given normal registration is full but both the selected Session and combined Event capacity have room When the Event Organiser manually adds an Attendee Then the registration is created as a distinguishable manual addition (C-58, T-50)
 Scenario 7 - Manual addition blocked at either limit
@@ -3422,7 +3422,7 @@
 - Keep an Attendee over-capacity submission Pending for Organiser review without counting it as an approved seat
 - Recheck both limits when the Organiser approves a Pending registration
 - Prevent concurrent requests from exceeding either limit
-- Offer the Event-level waiting list when combined Event capacity is full; keep a full selected Session on the Pending decision path with no Session-level waiting list (T-97)
+- Offer the Event-level waiting list when combined Event capacity is full; keep a full selected Session on the Pending decision path with no Session-level waiting list (T-98)
 - Allow manual VIP additions only within both limits and block them at either limit</t>
         </is>
       </c>
@@ -3431,7 +3431,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>C-05, C-58, C-78, C-98, T-30, T-31, T-50, T-85, B-11, T-97</t>
+          <t>C-05, C-58, C-78, C-98, T-30, T-31, T-50, T-85, B-11, T-98</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3520,7 +3520,7 @@
       <c r="F55" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Joined a full event's list
-Given the combined Event capacity is full and its Event-level waiting list is enabled When I join the waiting list Then I am added to the Event-level list and told I will be notified when a place is released; no Session-level waiting list is created (T-97)
+Given the combined Event capacity is full and its Event-level waiting list is enabled When I join the waiting list Then I am added to the Event-level list and told I will be notified when a place is released; no Session-level waiting list is created (T-98)
 Scenario 2 - Released place notified to all
 Given a place is released in an event with a waiting list When the place becomes available Then all waitlisted Attendees are notified and the place is claimed on a first-come, first-served basis
 Scenario 3 - Claimed place leaves the list
@@ -3541,7 +3541,7 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>C-23, T-33, T-46, B-10, T-97</t>
+          <t>C-23, T-33, T-46, B-10, T-98</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr"/>
@@ -4965,7 +4965,7 @@
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Previous event copied
-Given I choose one of my own completed or past events When I copy it Then ConnectSphere creates a new draft with the event requirements and Session structure copied, all event and Session dates/times left blank, and no bookings, reservations, or registrations carried over (T-98)
+Given I choose one of my own completed or past events When I copy it Then ConnectSphere creates a new draft with the event requirements and Session structure copied, all event and Session dates/times left blank, and no bookings, reservations, or registrations carried over (T-99)
 Scenario 2 - Missing reference flagged
 Given the copied event references a venue or equipment item that no longer exists When the draft is created Then the affected requirement is flagged for review and identifies its Session rather than being copied silently
 Scenario 3 - Dates remain subject to current submission policy
@@ -4973,7 +4973,7 @@
 Checklist
 - Copy one of my own completed or past events into a new draft
 - Confirm requirements and Session structure are copied while event and Session dates/times are blank
-- Confirm bookings, equipment reservations and registrations are not copied (T-98)
+- Confirm bookings, equipment reservations and registrations are not copied (T-99)
 - See unavailable venue/equipment references flagged against the relevant Session
 - Submit a copied draft subject to the current date rules</t>
         </is>
@@ -4983,7 +4983,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>C-74, T-79, T-87, T-90, T-98</t>
+          <t>C-74, T-79, T-87, T-90, T-99</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
@@ -7247,7 +7247,7 @@
 Scenario 4 - Concurrent submissions do not overbook
 Given one approved seat remains in a Session or in the combined Event capacity When two registrations are submitted at the same time Then at most one is confirmed against that remaining capacity and any other submission that exceeds capacity is Pending
 Scenario 5 - Waiting list remains event-level
-Given the combined Event capacity is full When an Attendee opens registration Then the existing Event-level waiting-list option is offered where enabled; a full selected Session follows the Pending decision path and has no separate Session-level waiting list (T-97)
+Given the combined Event capacity is full When an Attendee opens registration Then the existing Event-level waiting-list option is offered where enabled; a full selected Session follows the Pending decision path and has no separate Session-level waiting list (T-98)
 Scenario 6 - Manual addition allowed within both limits
 Given normal registration is full but both the selected Session and combined Event capacity have room When the Event Organiser manually adds an Attendee Then the registration is created as a distinguishable manual addition (C-58, T-50)
 Scenario 7 - Manual addition blocked at either limit
@@ -7258,7 +7258,7 @@
 - Keep an Attendee over-capacity submission Pending for Organiser review without counting it as an approved seat
 - Recheck both limits when the Organiser approves a Pending registration
 - Prevent concurrent requests from exceeding either limit
-- Offer the Event-level waiting list when combined Event capacity is full; keep a full selected Session on the Pending decision path with no Session-level waiting list (T-97)
+- Offer the Event-level waiting list when combined Event capacity is full; keep a full selected Session on the Pending decision path with no Session-level waiting list (T-98)
 - Allow manual VIP additions only within both limits and block them at either limit</t>
         </is>
       </c>
@@ -7267,7 +7267,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>C-05, C-58, C-78, C-98, T-30, T-31, T-50, T-85, B-11, T-97</t>
+          <t>C-05, C-58, C-78, C-98, T-30, T-31, T-50, T-85, B-11, T-98</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr"/>
@@ -7348,7 +7348,7 @@
       <c r="F64" s="2" t="inlineStr">
         <is>
           <t>Scenario 1 - Joined a full event's list
-Given the combined Event capacity is full and its Event-level waiting list is enabled When I join the waiting list Then I am added to the Event-level list and told I will be notified when a place is released; no Session-level waiting list is created (T-97)
+Given the combined Event capacity is full and its Event-level waiting list is enabled When I join the waiting list Then I am added to the Event-level list and told I will be notified when a place is released; no Session-level waiting list is created (T-98)
 Scenario 2 - Released place notified to all
 Given a place is released in an event with a waiting list When the place becomes available Then all waitlisted Attendees are notified and the place is claimed on a first-come, first-served basis
 Scenario 3 - Claimed place leaves the list
@@ -7369,7 +7369,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>C-23, T-33, T-46, B-10, T-97</t>
+          <t>C-23, T-33, T-46, B-10, T-98</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>

</xml_diff>